<commit_message>
Resolve KPI and model YAML through an optional kpi_group folder so authors can group configs without new ids.
Lookup stays by globally unique kpi_id / model_id across flat and one-level
group paths, so a KPI in one group can still point at a model in another.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KPI-Engine-Capabilities.xlsx
+++ b/docs/KPI-Engine-Capabilities.xlsx
@@ -312,8 +312,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Naming_conventions" displayName="Naming_conventions" ref="A1:E21" headerRowCount="1">
-  <autoFilter ref="A1:E21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Naming_conventions" displayName="Naming_conventions" ref="A1:E22" headerRowCount="1">
+  <autoFilter ref="A1:E22"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic"/>
     <tableColumn id="2" name="Convention"/>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Copy the pattern into config/kpis/&lt;id&gt;.yaml</t>
+          <t>Copy the pattern into config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1111,7 +1111,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Host entry: udfs.kpi_engine.main   |   Routing: execution.kpi_id → config/kpis/&lt;id&gt;.yaml   |   AI brief: attach YAML preparation + catalogs + calculation intake (kpi-yaml-preparation-guide.md §0).</t>
+          <t>Host entry: udfs.kpi_engine.main   |   Routing: execution.kpi_id → config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml   |   AI brief: attach YAML preparation + catalogs + calculation intake (kpi-yaml-preparation-guide.md §0).</t>
         </is>
       </c>
     </row>
@@ -6647,12 +6647,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Copy config/kpis/3004.yaml → &lt;kpi_id&gt;.yaml. Fill time, dimensions, base_measures, cuts, measures. Host module_path stays udfs.kpi_engine.main.</t>
+          <t>Copy config/kpis/sotif/3004.yaml → &lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml. Fill time, dimensions, base_measures, cuts, measures. Host module_path stays udfs.kpi_engine.main.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>udfs/config/kpis/&lt;id&gt;.yaml</t>
+          <t>udfs/config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -6674,12 +6674,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Add config/models/&lt;id&gt;.yaml (kind: physical or sql). Point KPI model: at model_id. Paths stay on context.datasets.</t>
+          <t>Add config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml (kind: physical or sql). Point KPI model: at model_id. Paths stay on context.datasets.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>udfs/config/models/&lt;id&gt;.yaml</t>
+          <t>udfs/config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -6979,7 +6979,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>config/kpis/&lt;kpi_id&gt;.yaml</t>
+          <t>config/kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml (or flat kpis/&lt;kpi_id&gt;.yaml)</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>config/models/&lt;id&gt;.yaml  —  KPI model: pointer</t>
+          <t>config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml  —  KPI model: pointer</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -7445,7 +7445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7490,534 +7490,561 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Path is exact: udfs/config/kpis/&lt;kpi_id&gt;.yaml. The stem must equal context.execution.kpi_id with no name-fold.</t>
+          <t>Path: udfs/config/kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml or flat kpis/&lt;kpi_id&gt;.yaml. Stem equals execution.kpi_id exactly (no fold). kpi_id is unique across groups.</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>3004.yaml when execution.kpi_id is 3004 or "3004". Copy 3004.yaml to &lt;new_id&gt;.yaml.</t>
+          <t>kpis/sotif/3004.yaml when execution.kpi_id is 3004. Copy to kpis/&lt;kpi_group&gt;/&lt;new_id&gt;.yaml.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>sotif.yaml for kpi_id 3004. 3004.yml. kpis/Sotif.yaml when the host sends 3004. Spaces or extra folders.</t>
+          <t>sotif.yaml for kpi_id 3004. 3004.yml. Two groups both containing 3004.yaml. kpis/sotif/quality/3004.yaml (only one group folder).</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>load_kpi opens only f"{kpi_id}.yaml". A missing file is a bind error. Case on the filename is OS-dependent; treat it as exact.</t>
+          <t>load_kpi finds exactly one f"{kpi_id}.yaml" under kpis/ or kpis/*/. Zero or two files is a bind error. No execution.kpi_group field.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="29" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>KPI yaml kpi_id:</t>
+          <t>kpi_group folder</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Set kpi_id: to the same value as the filename stem (and the host execution.kpi_id).</t>
+          <t>One optional snake_case directory under kpis/ and models/. Authoring only; not sent on the context. Group names use the identifier alphabet.</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>File 3004.yaml → kpi_id: 3004. File freight_fill.yaml → kpi_id: freight_fill.</t>
+          <t>kpis/sotif/, models/sotif/, models/freight/. A KPI in kpis/sotif/ may model: a file in models/freight/.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>File 3004.yaml with kpi_id: sotif. Reusing one YAML for several ids.</t>
+          <t>execution.kpi_group. Nested groups (kpis/a/b/id.yaml). Spaces or hyphens in the folder name.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>The engine loads by filename. Inner kpi_id: is the spec id; keep it identical so logs and errors match the request.</t>
+          <t>The engine never reads the folder name. Duplicate kpi_id or model_id across groups is a bind error.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="29" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Model YAML file</t>
+          <t>KPI yaml kpi_id:</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Path: udfs/config/models/&lt;model_id&gt;.yaml. Prefer lowercase snake_case. Extension must be .yaml.</t>
+          <t>Set kpi_id: to the same value as the filename stem (and the host execution.kpi_id).</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>sotif.yaml, orders_sql.yaml, freight_lane.yaml.</t>
+          <t>File 3004.yaml → kpi_id: 3004. File freight_fill.yaml → kpi_id: freight_fill.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>sotif.yml. models/Sotif Model.yaml. Putting the file under kpis/.</t>
+          <t>File 3004.yaml with kpi_id: sotif. Reusing one YAML for several ids.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>load_model first tries &lt;model_id&gt;.yaml exactly. If missing, it accepts exactly one *.yaml whose stem folds to model_id (Sotif.yaml ↔ sotif). Two fold-matches is an error.</t>
+          <t>The engine loads by filename. Inner kpi_id: is the spec id; keep it identical so logs and errors match the request.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="29" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Model yaml model_id:</t>
+          <t>Model YAML file</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>model_id: must equal the filename stem you intend KPIs to point at. Prefer the same spelling everywhere.</t>
+          <t>Path: udfs/config/models/&lt;kpi_group&gt;/&lt;model_id&gt;.yaml or flat models/&lt;model_id&gt;.yaml. Prefer lowercase snake_case. Extension must be .yaml. model_id is unique across groups.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>File sotif.yaml → model_id: sotif. File orders_sql.yaml → model_id: orders_sql.</t>
+          <t>models/sotif/sotif.yaml, models/freight/orders_sql.yaml.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>File sotif.yaml with model_id: sotif_sql. Two files that fold to the same id.</t>
+          <t>sotif.yml. models/Sotif Model.yaml. Two groups both containing sotif.yaml. Putting the file under kpis/.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>KPI model: is matched to this field after folding case / spaces / underscores. Extra tokens do not fold away: sotif ≠ sotif_sql.</t>
+          <t>load_model finds exactly one file whose stem folds to model_id among models/*.yaml and models/*/*.yaml (Sotif.yaml ↔ sotif). Two fold-matches is an error.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="29" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>KPI model: pointer</t>
+          <t>Model yaml model_id:</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>KPI YAML model: must name a model_id that exists. Same fold as model_id (case, spaces, underscores only).</t>
+          <t>model_id: must equal the filename stem you intend KPIs to point at. Prefer the same spelling everywhere.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>model: sotif  with models/sotif.yaml. Per-base override base_measures.x.model: orders_sql when two extracts are needed.</t>
+          <t>File sotif.yaml → model_id: sotif. File orders_sql.yaml → model_id: orders_sql.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>model: sotif pointing at sotif_sql.yaml. Embedding an ADLS path instead of a model id. Inventing a model that has no file.</t>
+          <t>File sotif.yaml with model_id: sotif_sql. Two files that fold to the same id.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>same_model_id folds Region/region and my_model/my model. It does not treat sotif as sotif_sql. Physical vs sql is kind: on the model file, not a suffix rule — but keep suffixes honest (orders_sql.yaml for kind: sql).</t>
+          <t>KPI model: is matched to this field after folding case / spaces / underscores. Extra tokens do not fold away: sotif ≠ sotif_sql.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="29" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Identifier alphabet</t>
+          <t>KPI model: pointer</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>YAML names that become SQL/Pandas identifiers must match ^[A-Za-z_][A-Za-z0-9_]*$. Prefer snake_case.</t>
+          <t>KPI YAML model: must name a model_id that exists. Same fold as model_id (case, spaces, underscores only).</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>reason_code, current_value, event_month, sotif_value, shipped_now.</t>
+          <t>model: sotif  with models/sotif/sotif.yaml (or models/freight/sotif.yaml). Per-base override base_measures.x.model: orders_sql when two extracts are needed.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>reason-code, reason.code, "Reason Code", 12m_trend, current value.</t>
+          <t>model: sotif pointing at sotif_sql.yaml. Embedding an ADLS path instead of a model id. Inventing a model that has no file.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>require_ident rejects hyphens, dots, spaces, quotes, and leading digits. Used for dimensions, base_measures, parameters, aliases, sources, join keys, time.column, filter_map values, output_schema, columns: lists.</t>
+          <t>same_model_id folds Region/region and my_model/my model. It does not treat sotif as sotif_sql. Physical vs sql is kind: on the model file, not a suffix rule — but keep suffixes honest (orders_sql.yaml for kind: sql).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="29" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Reserved words in formulas</t>
+          <t>Identifier alphabet</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Do not use these as column or measure names inside expr: / CASE: case, when, then, else, and, or, not, is, null, in.</t>
+          <t>YAML names that become SQL/Pandas identifiers must match ^[A-Za-z_][A-Za-z0-9_]*$. Prefer snake_case.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>date_diff(start, end, 'day') — end is legal. Names like region, amount, shipped_now.</t>
+          <t>reason_code, current_value, event_month, sotif_value, shipped_now.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>expr: case / qty. A column named when or in.</t>
+          <t>reason-code, reason.code, "Reason Code", 12m_trend, current value.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Parser treats those as CASE/boolean keywords. end is a CASE terminator but is allowed as an identifier (date_diff(start, end, 'day')).</t>
+          <t>require_ident rejects hyphens, dots, spaces, quotes, and leading digits. Used for dimensions, base_measures, parameters, aliases, sources, join keys, time.column, filter_map values, output_schema, columns: lists.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="29" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Name folding (host ↔ YAML)</t>
+          <t>Reserved words in formulas</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Host keys fold onto YAML keys: lowercase, trim, spaces → underscore. Measure keys also try a compact fold (drop remaining underscores).</t>
+          <t>Do not use these as column or measure names inside expr: / CASE: case, when, then, else, and, or, not, is, null, in.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>YAML current_value matches host Current_Value or current value. YAML previous_year_value matches PreviousYearValue.</t>
+          <t>date_diff(start, end, 'day') — end is legal. Names like region, amount, shipped_now.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Relying on fold for file names (KPI files do not fold). Expecting sotif to match sotif_sql. Two YAML keys that fold to the same spelling.</t>
+          <t>expr: case / qty. A column named when or in.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>norm_name is case/space/underscore only. Use one canonical snake_case in YAML; the host may send UI Title Case. Do not create two keys that collide after fold.</t>
+          <t>Parser treats those as CASE/boolean keywords. end is a CASE terminator but is allowed as an identifier (date_diff(start, end, 'day')).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="29" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Measure keys</t>
+          <t>Name folding (host ↔ YAML)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Keys under measures: are what context.measures_required[].measure_key must match (after fold). snake_case. Must not collide with parameters.</t>
+          <t>Host keys fold onto YAML keys: lowercase, trim, spaces → underscore. Measure keys also try a compact fold (drop remaining underscores).</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>current_value, previous_year_value, trailing_3m, yoy_pct, fill_rate.</t>
+          <t>YAML current_value matches host Current_Value or current value. YAML previous_year_value matches PreviousYearValue.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Current Value as the YAML key. Reusing a parameter name. A key that is not in the host contract.</t>
+          <t>Relying on fold for file names (KPI files do not fold). Expecting sotif to match sotif_sql. Two YAML keys that fold to the same spelling.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Unknown measure_key is a bind error listing valid YAML keys. An empty measures_required list computes nothing (it does not expand to every key).</t>
+          <t>norm_name is case/space/underscore only. Use one canonical snake_case in YAML; the host may send UI Title Case. Do not create two keys that collide after fold.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="29" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Base measure names</t>
+          <t>Measure keys</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Keys under base_measures: are internal facts. UI does not request these names. snake_case identifiers.</t>
+          <t>Keys under measures: are what context.measures_required[].measure_key must match (after fold). snake_case. Must not collide with parameters.</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>sotif_value, shipped_qty, ordered_qty, line_rev.</t>
+          <t>current_value, previous_year_value, trailing_3m, yoy_pct, fill_rate.</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Naming a base the same as a requestable measure unless you intend identity. Hyphenated names.</t>
+          <t>Current Value as the YAML key. Reusing a parameter name. A key that is not in the host contract.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Measures reference bases via of:. A base with no agg: is a row helper, not a requestable point.</t>
+          <t>Unknown measure_key is a bind error listing valid YAML keys. An empty measures_required list computes nothing (it does not expand to every key).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="29" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Dimensions</t>
+          <t>Base measure names</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Catalog names under dimensions[].name (and from: if the physical column differs). Request selected_dimensions must pick from this allowlist.</t>
+          <t>Keys under base_measures: are internal facts. UI does not request these names. snake_case identifiers.</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>- { name: supplier, from: supplier_name }. default_dimensions: [reason_code].</t>
+          <t>sotif_value, shipped_qty, ordered_qty, line_rev.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Inventing a request dimension not in YAML. Using the host display label as the YAML name when the column is supplier_name (map it with from:).</t>
+          <t>Naming a base the same as a requestable measure unless you intend identity. Hyphenated names.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>YAML owns the allowlist. from: is the physical/model column; name: is the grain token the request uses.</t>
+          <t>Measures reference bases via of:. A base with no agg: is a row helper, not a requestable point.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="29" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Cut names</t>
+          <t>Dimensions</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Short stable tokens. G and R in 3004 are examples, not engine-hardcoded. default_cut must be one of the declared names.</t>
+          <t>Catalog names under dimensions[].name (and from: if the physical column differs). Request selected_dimensions must pick from this allowlist.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>cuts: [{ name: G, … }, { name: R, group_by: [region] }]. default_cut: G.</t>
+          <t>- { name: supplier, from: supplier_name }. default_dimensions: [reason_code].</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Renaming G/R in YAML without updating the host cut list. Two cuts with the same name.</t>
+          <t>Inventing a request dimension not in YAML. Using the host display label as the YAML name when the column is supplier_name (map it with from:).</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Cut name is a string the host sends; group_by entries must be catalog dimensions (identifiers). Also_emit / ignore_filters name other cuts or filter codes.</t>
+          <t>YAML owns the allowlist. from: is the physical/model column; name: is the grain token the request uses.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>Cut names</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Short stable tokens. G and R in 3004 are examples, not engine-hardcoded. default_cut must be one of the declared names.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>cuts: [{ name: G, … }, { name: R, group_by: [region] }]. default_cut: G.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Renaming G/R in YAML without updating the host cut list. Two cuts with the same name.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Cut name is a string the host sends; group_by entries must be catalog dimensions (identifiers). Also_emit / ignore_filters name other cuts or filter codes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="29" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>Dataset aliases</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>model.required_aliases and sources.*.alias must be identifiers. They bind to context.datasets by alias or key, case-insensitive.</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>required_aliases: [sotif]. Host dataset alias or key: sotif (or SOTIF).</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>required_aliases: [my-table]. Putting an ADLS URI in the alias. A KPI-level path instead of an alias.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Context path wins; model default_path / default_paths fills gaps. Do not put dataset URIs in KPI YAML.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>SQL model placeholders</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>kind: sql models reference bound datasets as $alias_path or $alias_scan (alias = required_aliases entry).</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>sql: |
   SELECT … FROM $sotif_scan WHERE …</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Hard-coding /mnt/… or abfss:// in the SQL. Using an alias that is not in required_aliases.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>$alias_scan becomes delta_scan(?) or read_parquet(?) from table_type. $alias_path is the path parameter. Order of placeholders must match bind order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="29" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Time grains</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Only: day, week, month, quarter, year (lowercase). Default grain is month.</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>time: { column: event_month, grain: month, filter_code: reporting_month }.</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>time.grain: monthly. MTD as a grain name. execution.time_grain on the host payload.</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Send parameters.time_grain when the KPI declares that parameter. execution.time_grain is rejected. calendar: gregorian or fiscal.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="29" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>time.filter_code and filter_map keys</t>
+          <t>Time grains</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>These are host filter codes, not SQL identifiers. They may contain spaces. filter_map values (columns) must still be identifiers.</t>
+          <t>Only: day, week, month, quarter, year (lowercase). Default grain is month.</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>filter_code: reporting_month. filter_map: { "Supplier Name": supplier_name }.</t>
+          <t>time: { column: event_month, grain: month, filter_code: reporting_month }.</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>filter_map values with spaces or hyphens. Omitting filter_code when time: is present.</t>
+          <t>time.grain: monthly. MTD as a grain name. execution.time_grain on the host payload.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>time.filter_code is required when time: is declared. It names the context filter that carries the selected period (the anchor), not a month IN list.</t>
+          <t>Send parameters.time_grain when the KPI declares that parameter. execution.time_grain is rejected. calendar: gregorian or fiscal.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="29" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Parameters</t>
+          <t>time.filter_code and filter_map keys</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Parameter names are identifiers. Must not equal a measure key. Do not declare selected_dimensions as a parameter. when: case labels cannot be param, cases, or else.</t>
+          <t>These are host filter codes, not SQL identifiers. They may contain spaces. filter_map values (columns) must still be identifiers.</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>parameters: { time_grain: { type: string, allowed: [month, quarter] } }.</t>
+          <t>filter_code: reporting_month. filter_map: { "Supplier Name": supplier_name }.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>parameters.selected_dimensions. A case label named else. A parameter named current_value when that is also a measure key.</t>
+          <t>filter_map values with spaces or hyphens. Omitting filter_code when time: is present.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>time_grain is the reserved overlay formerly on execution. Case labels param / cases / else are when: metadata keys.</t>
+          <t>time.filter_code is required when time: is declared. It names the context filter that carries the selected period (the anchor), not a month IN list.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="29" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Host UDF / module_path</t>
+          <t>Parameters</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>One generic entry: udfs.kpi_engine.main. Routing is execution.kpi_id → config/kpis/&lt;id&gt;.yaml. Do not add a per-KPI Python module.</t>
+          <t>Parameter names are identifiers. Must not equal a measure key. Do not declare selected_dimensions as a parameter. when: case labels cannot be param, cases, or else.</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Host module_path: udfs.kpi_engine.main. New KPI = new YAML (+ model YAML if the extract is new).</t>
+          <t>parameters: { time_grain: { type: string, allowed: [month, quarter] } }.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>udfs/&lt;kpi_id&gt;/main.py. Cloning the engine per metric. A second module_path per kpi_id.</t>
+          <t>parameters.selected_dimensions. A case label named else. A parameter named current_value when that is also a measure key.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>The UDF is stateless compute(context). KPI math lives in YAML; DuckDB shape lives in model YAML.</t>
+          <t>time_grain is the reserved overlay formerly on execution. Case labels param / cases / else are when: metadata keys.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="29" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>What must not live in KPI YAML</t>
+          <t>Host UDF / module_path</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>No dataset URIs, no Python, no invented op:/hook:/fn: names, no per-cut model:.</t>
+          <t>One generic entry: udfs.kpi_engine.main. Routing is execution.kpi_id → config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml (or flat kpis/&lt;id&gt;.yaml). Do not add a per-KPI Python module.</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>model: sotif. op: point / window / rank / hook / expr — names from this workbook's catalogs.</t>
+          <t>Host module_path: udfs.kpi_engine.main. New KPI = new YAML (+ model YAML if the extract is new).</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>abfss://… in the KPI file. op: my_custom_yoy. cuts: [{ model: other }]. A sibling .py next to the YAML.</t>
+          <t>udfs/&lt;kpi_id&gt;/main.py. Cloning the engine per metric. A second module_path per kpi_id.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Paths belong on context.datasets or model default_paths. Catalog names are the Measure ops / Functions / Hooks sheets. cuts cannot set model:.</t>
+          <t>The UDF is stateless compute(context). KPI math lives in YAML; DuckDB shape lives in model YAML.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="29" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>What must not live in KPI YAML</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>No dataset URIs, no Python, no invented op:/hook:/fn: names, no per-cut model:.</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>model: sotif. op: point / window / rank / hook / expr — names from this workbook's catalogs.</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>abfss://… in the KPI file. op: my_custom_yoy. cuts: [{ model: other }]. A sibling .py next to the YAML.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Paths belong on context.datasets or model default_paths. Catalog names are the Measure ops / Functions / Hooks sheets. cuts cannot set model:.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="29" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>File header comments (recommended)</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Match existing config files: what the file provides, where it is used, capabilities, when to copy it.</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>See udfs/config/kpis/3004.yaml and udfs/config/models/sotif.yaml headers.</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>See udfs/config/kpis/sotif/3004.yaml and udfs/config/models/sotif/sotif.yaml headers.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Leaving a copied file with the old kpi_id / Sotif description. Putting secrets in comments.</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Comments are documentation only; the engine ignores them. Keep kpi_id / model_id in the body in sync with the filename.</t>
         </is>
@@ -8109,7 +8136,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Every generating response is: (1) entire kpis/&lt;kpi_id&gt;.yaml (2) entire models/&lt;model_id&gt;.yaml if extract is new, else 'reuses existing model' (3) Assumptions (4) Gaps.</t>
+          <t>Every generating response is: (1) entire kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml (2) entire models/&lt;kpi_group&gt;/&lt;model_id&gt;.yaml if extract is new, else 'reuses existing model' (3) Assumptions (4) Gaps.</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -8468,7 +8495,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>See gold file udfs/config/kpis/3004.yaml — copy structure, not Sotif names, unless this KPI is Sotif.</t>
+          <t>See gold file udfs/config/kpis/sotif/3004.yaml — copy structure, not Sotif names, unless this KPI is Sotif.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Close the count, where, and composite time-shift gaps real-world KPI tests exposed.
Text count no longer silently returns zero, numeric where: compares bind, and lag/diff of fn/expr/window composites evaluate at the shifted anchor instead of the request month.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KPI-Engine-Capabilities.xlsx
+++ b/docs/KPI-Engine-Capabilities.xlsx
@@ -270,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="All_operations" displayName="All_operations" ref="A1:E29" headerRowCount="1">
-  <autoFilter ref="A1:E29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="All_operations" displayName="All_operations" ref="A1:E30" headerRowCount="1">
+  <autoFilter ref="A1:E30"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Operation"/>
@@ -326,8 +326,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="YAML_preparation" displayName="YAML_preparation" ref="A1:E22" headerRowCount="1">
-  <autoFilter ref="A1:E22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="YAML_preparation" displayName="YAML_preparation" ref="A1:E24" headerRowCount="1">
+  <autoFilter ref="A1:E24"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic"/>
     <tableColumn id="2" name="What to provide / emit"/>
@@ -5240,7 +5240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5361,25 +5361,29 @@
     <row r="5" ht="29" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Aggregation</t>
+          <t>Row helper</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>min / max</t>
+          <t>where:</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Recomputed at every cut (not summed regional extrema).</t>
+          <t>Pandas row mask before fold. Numeric ops coerce the compare column. ne excludes nulls (SQL-style).</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>base_measures.peak: { sql: amount, agg: max }</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr"/>
+          <t>where: { column: mrr, op: gt, value: 0 }</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Ops: in eq ne gt gte lt lte between. between needs values: [lo, hi]. Not like/is_null.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="29" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -5389,24 +5393,20 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>count_distinct</t>
+          <t>min / max</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Distinct values. Non-additive; re-reads row-level detail.</t>
+          <t>Recomputed at every cut (not summed regional extrema).</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>base_measures.n: { sql: order_id, agg: count_distinct }</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Not folded in DuckDB GROUP BY</t>
-        </is>
-      </c>
+          <t>base_measures.peak: { sql: amount, agg: max }</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="29" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -5416,22 +5416,22 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>median / percentile</t>
+          <t>count_distinct</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Non-additive. percentile requires percentile: 0–100.</t>
+          <t>Distinct values. Non-additive; re-reads row-level detail.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>base_measures.p90: { sql: amount, agg: percentile, percentile: 90 }</t>
+          <t>base_measures.n: { sql: order_id, agg: count_distinct }</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Row-level path</t>
+          <t>Not folded in DuckDB GROUP BY</t>
         </is>
       </c>
     </row>
@@ -5443,49 +5443,49 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>first / last</t>
+          <t>median / percentile</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Identity fold after sort by time (or window).</t>
+          <t>Non-additive. percentile requires percentile: 0–100.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>base_measures.bal: { sql: balance, agg: last }</t>
+          <t>base_measures.p90: { sql: amount, agg: percentile, percentile: 90 }</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Used with over: last_n</t>
+          <t>Row-level path</t>
         </is>
       </c>
     </row>
     <row r="9" ht="29" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Row helper</t>
+          <t>Aggregation</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>expr</t>
+          <t>first / last</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Named row formula on columns or earlier helpers. No DuckDB SUM().</t>
+          <t>Identity fold after sort by time (or window). Text columns are still coerced to numeric.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>gross: { expr: qty * price }</t>
+          <t>base_measures.bal: { sql: balance, agg: last }</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Add agg: to fold, or identity_grain for point of</t>
+          <t>Used with over: last_n</t>
         </is>
       </c>
     </row>
@@ -5497,20 +5497,24 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>lookup</t>
+          <t>expr</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Map a column through a dict; default or strict.</t>
+          <t>Named row formula on columns or earlier helpers. No DuckDB SUM().</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>fee: { lookup: { column: pay, map: { COD: 25 }, default: 10 } }</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>gross: { expr: qty * price }</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Add agg: to fold, or identity_grain for point of</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="29" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -5520,17 +5524,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>sql: column</t>
+          <t>lookup</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Pass a physical column (or simple ident). Default agg is sum if omitted.</t>
+          <t>Map a column through a dict; default or strict.</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>sotif_value: { sql: amount, agg: sum }</t>
+          <t>fee: { lookup: { column: pay, map: { COD: 25 }, default: 10 } }</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
@@ -5543,49 +5547,45 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>columns + op</t>
+          <t>sql: column</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Call a column function by name.</t>
+          <t>Pass a physical column (or simple ident). Default agg is sum if omitted.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>ontime_full: { columns: [ontime, fullqty], op: multiply, agg: sum }</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>See Column functions sheet</t>
-        </is>
-      </c>
+          <t>sotif_value: { sql: amount, agg: sum }</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="29" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Entity window</t>
+          <t>Row helper</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>over.lag / lead</t>
+          <t>columns + op</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Value from another row in partition, ordered by order_by. Requires of:.</t>
+          <t>Call a column function by name.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>prev: { over: { fn: lag, of: order_date, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
+          <t>ontime_full: { columns: [ontime, fullqty], op: multiply, agg: sum }</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Not calendar op: lag</t>
+          <t>See Column functions sheet</t>
         </is>
       </c>
     </row>
@@ -5597,20 +5597,24 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>over.row_number / rank / dense_rank</t>
+          <t>over.lag / lead</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Sequence in partition. of: optional.</t>
+          <t>Value from another row in partition, ordered by order_by. Requires of:.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>seq: { over: { fn: row_number, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>prev: { over: { fn: lag, of: order_date, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Not calendar op: lag</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -5620,17 +5624,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>over.running_sum / running_avg</t>
+          <t>over.row_number / rank / dense_rank</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Running aggregate along order_by. Requires of:.</t>
+          <t>Sequence in partition. of: optional.</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>run: { over: { fn: running_sum, of: net, partition_by: [carrier_id], order_by: [start] }, agg: max }</t>
+          <t>seq: { over: { fn: row_number, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
@@ -5643,49 +5647,45 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>over.last_n</t>
+          <t>over.running_sum / running_avg</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>JSON list of last n of values. Point only; cannot feed arithmetic.</t>
+          <t>Running aggregate along order_by. Requires of:.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>recent: { over: { fn: last_n, of: amount, n: 2, partition_by: [region], order_by: [order_id] }, agg: last }</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Dates as ISO strings</t>
-        </is>
-      </c>
+          <t>run: { over: { fn: running_sum, of: net, partition_by: [carrier_id], order_by: [start] }, agg: max }</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="29" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Entity window</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>grain day/week/month/quarter/year</t>
+          <t>over.last_n</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Bucket of the time column. Fiscal calendar only for Q/Y.</t>
+          <t>JSON list of last n of values. Point only; cannot feed arithmetic.</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>time: { column: event_month, grain: month, filter_code: reporting_month }</t>
+          <t>recent: { over: { fn: last_n, of: amount, n: 2, partition_by: [region], order_by: [order_id] }, agg: last }</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>parameters.time_grain overlay if declared</t>
+          <t>Dates as ISO strings</t>
         </is>
       </c>
     </row>
@@ -5697,20 +5697,24 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>point offset</t>
+          <t>grain day/week/month/quarter/year</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Same measure at calendar offset from anchor.</t>
+          <t>Bucket of the time column. Fiscal calendar only for Q/Y.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>previous_year_value: { of: sotif_value, op: point, offset: { years: 1 } }</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr"/>
+          <t>time: { column: event_month, grain: month, filter_code: reporting_month }</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>parameters.time_grain overlay if declared</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="29" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -5720,17 +5724,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>window trailing / leading</t>
+          <t>point offset</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Inclusive trailing N (or leading) periods as one number.</t>
+          <t>Same measure at calendar offset from anchor.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>value_3m: { of: sotif_value, op: window, trailing: { months: 3 }, inclusive: true }</t>
+          <t>previous_year_value: { of: sotif_value, op: point, offset: { years: 1 } }</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -5743,24 +5747,20 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>window range</t>
+          <t>window trailing / leading</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ytd, qtd, mtd, wtd, cumulative, full_month/quarter/year.</t>
+          <t>Inclusive trailing N (or leading) periods as one number.</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>value_qtd: { of: sotif_value, op: window, range: qtd }</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>wtd needs day grain</t>
-        </is>
-      </c>
+          <t>value_3m: { of: sotif_value, op: window, trailing: { months: 3 }, inclusive: true }</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
     </row>
     <row r="21" ht="29" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -5770,22 +5770,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>trend</t>
+          <t>window range</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Fixed-length array + trend_axes / trend_labels. Cap 50,000 cells/cut.</t>
+          <t>ytd, qtd, mtd, wtd, cumulative, full_month/quarter/year.</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>trend_12m: { of: sotif_value, op: trend, trailing: { months: 12 } }</t>
+          <t>value_qtd: { of: sotif_value, op: window, range: qtd }</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Defaults to default_cut only</t>
+          <t>wtd needs day grain</t>
         </is>
       </c>
     </row>
@@ -5797,49 +5797,49 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>snapshot (omit time:)</t>
+          <t>trend</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>No month filter; all matching rows. Host reporting_month skipped as no_time.</t>
+          <t>Fixed-length array + trend_axes / trend_labels. Cap 50,000 cells/cut.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Omit the time: block; only point offset 0 (and constants).</t>
+          <t>trend_12m: { of: sotif_value, op: trend, trailing: { months: 12 } }</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>No windows/trends/nonzero offsets</t>
+          <t>Defaults to default_cut only</t>
         </is>
       </c>
     </row>
     <row r="23" ht="29" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Cuts</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>group_by / ignore_filters / also_emit</t>
+          <t>snapshot (omit time:)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Named grains. G/R are examples, not hardcoded.</t>
+          <t>No month filter; all matching rows. Host reporting_month skipped as no_time.</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>cuts: [{ name: G, group_by: [], ignore_filters: [region], also_emit: [R] }]</t>
+          <t>Omit the time: block; only point offset 0 (and constants).</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>selected_dimensions overlays request grain</t>
+          <t>No windows/trends/nonzero offsets</t>
         </is>
       </c>
     </row>
@@ -5851,22 +5851,22 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>having</t>
+          <t>group_by / ignore_filters / also_emit</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Drop groups that fail measure predicates. Optional then_group_by.</t>
+          <t>Named grains. G/R are examples, not hardcoded.</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>having: { predicates: [{ of: current_value, cmp: gt, value: 0 }] }</t>
+          <t>cuts: [{ name: G, group_by: [], ignore_filters: [region], also_emit: [R] }]</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>cmp: gt gte lt lte eq ne between</t>
+          <t>selected_dimensions overlays request grain</t>
         </is>
       </c>
     </row>
@@ -5878,124 +5878,151 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>green_when</t>
+          <t>having</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Boolean green flag on survivors (above/below).</t>
+          <t>Drop groups that fail measure predicates. Optional then_group_by.</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>green_when: { of: current_value, above: 40 }</t>
+          <t>having: { predicates: [{ of: current_value, cmp: gt, value: 0 }] }</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Does not drop rows</t>
+          <t>cmp: gt gte lt lte eq ne between</t>
         </is>
       </c>
     </row>
     <row r="26" ht="29" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Cuts</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>apply extract / calc / result</t>
+          <t>green_when</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>DuckDB WHERE vs Pandas vs drop JSON rows.</t>
+          <t>Boolean green flag on survivors (above/below).</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>filters: { region: { apply: extract } }</t>
+          <t>green_when: { of: current_value, above: 40 }</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Unmapped valued filters are FilterError</t>
+          <t>Does not drop rows</t>
         </is>
       </c>
     </row>
     <row r="27" ht="29" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Multi-model</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>model_relations</t>
+          <t>apply extract / calc / result</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Join two extracts on declared keys.</t>
+          <t>DuckDB WHERE vs Pandas vs drop JSON rows.</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>model_relations: [{ left: a, right: b, on: [event_month, region], how: left }]</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr"/>
+          <t>filters: { region: { apply: extract } }</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Unmapped valued filters are FilterError</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="29" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Multi-model</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>identity_grain</t>
+          <t>model_relations</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Helpers as measures.of only when every emitted cut equals this grain.</t>
+          <t>Join two extracts on declared keys.</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>identity_grain: [carrier_id, shipment_id]</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Otherwise BindError; fold with agg:</t>
-        </is>
-      </c>
+          <t>model_relations: [{ left: a, right: b, on: [event_month, region], how: left }]</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
     </row>
     <row r="29" ht="29" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>identity_grain</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Helpers as measures.of only when every emitted cut equals this grain.</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>identity_grain: [carrier_id, shipment_id]</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Otherwise BindError; fold with agg:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="29" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>SQL model</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>kind: sql</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Shape extract with CTEs; walked columns must be in output_schema.</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>models/&lt;id&gt;.yaml kind: sql + sql: + output_schema:</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Not KPI sql: formulas</t>
         </is>
@@ -8064,7 +8091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8322,350 +8349,406 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>Map — last period of a composite</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Lag/diff/index of a ratio, OEE, or rolling window — not a duplicated prior_* subgraph.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>prior_oee: { op: lag, of: oee_pct, offset: { months: 1 } }
+delta: { op: diff, of: oee_pct, offset: { months: 1 } }</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>lag of trend/hook/rank. lag of a row helper (no agg:).</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Sources: bases and shiftable measures (point, window, fn, expr, …).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Map — row mask (where:)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>COUNT/SUM only the rows that pass a comparison (status, mrr &gt; 0, amount between).</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>where: { column: mrr, op: gt, value: 0 }
+between: { column: amount, op: between, values: [lo, hi] }</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>like / is_null on base where:. between with only value:.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Ops: in eq ne gt gte lt lte between. ne excludes nulls (SQL-style). Numeric ops coerce the column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>Map — trailing N / YTD / QTD</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Trailing N periods as one number; or named period-to-date.</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>value_3m: { of: fact, op: window, trailing: { months: 3 }, inclusive: true }
 value_qtd: { of: fact, op: window, range: qtd }</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Summing three point keys. range: qtd to mean trailing 3. wtd at month grain.</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>range: trailing | leading | cumulative | ytd | mtd | qtd | wtd | full_month | full_quarter | full_year. wtd needs day grain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="29" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Map — graph / trend</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Last N periods as an array for a chart.</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>trend_12m: { of: fact, op: trend, trailing: { months: 12 }, cuts: [G] }</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Returning N point keys. Unrestricted trend on a high-cardinality cut (50k cell cap).</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Trend defaults to default_cut if cuts: omitted. Axis lands in response trend_axes / trend_labels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="29" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Map — ratio of totals vs sum of ratios</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Fill rate / rate KPIs: decide per-row then SUM vs SUM/SUM.</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Two summed bases → two points → measures.fill_rate: { op: expr, expr: shipped_now / ordered_now }</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>base expr shipped/ordered + agg: sum when the spec wanted ratio of totals.</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>base expr identifiers are physical columns. measure expr identifiers are other measure keys. Do not mix expr: with columns:/op:/sql: on one base.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="29" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Map — share / rank / SLA</t>
+          <t>Map — graph / trend</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Share of all groups on this cut; rank; hit-rate over a series.</t>
+          <t>Last N periods as an array for a chart.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>op: percent_of_total (not fn: percent). op: rank. op: hook + hook: hit_rate + trailing: + value:.</t>
+          <t>trend_12m: { of: fact, op: trend, trailing: { months: 12 }, cuts: [G] }</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>fn: percent for cut share. Sorting in the host to fake rank. A window SUM for 'how often'.</t>
+          <t>Returning N point keys. Unrestricted trend on a high-cardinality cut (50k cell cap).</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Cut ops see the full cut. Hooks need the densified spine — declare trailing so required_span is wide enough.</t>
+          <t>Trend defaults to default_cut if cuts: omitted. Axis lands in response trend_axes / trend_labels.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Map — snapshot / entity window / lookup</t>
+          <t>Map — ratio of totals vs sum of ratios</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>No period column; per-entity sequence; static code map.</t>
+          <t>Fill rate / rate KPIs: decide per-row then SUM vs SUM/SUM.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Omit time:. over: on a pre-fold base (not calendar op: lag). lookup: { column, map, default }.</t>
+          <t>Two summed bases → two points → measures.fill_rate: { op: expr, expr: shipped_now / ordered_now }</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>window/trend on a snapshot. Calendar op: lag for per-customer previous order. Giant CASE for a fee table.</t>
+          <t>base expr shipped/ordered + agg: sum when the spec wanted ratio of totals.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Snapshot leftover reporting_month skips as no_time. identity_grain required to point at a helper with no agg:.</t>
+          <t>base expr identifiers are physical columns. measure expr identifiers are other measure keys. Do not mix expr: with columns:/op:/sql: on one base.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Map — cannot express</t>
+          <t>Map — share / rank / SLA</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Iterative allocation, custom solver, anything with no catalog row.</t>
+          <t>Share of all groups on this cut; rank; hit-rate over a series.</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Stop. Report: cannot bind with current catalog. Name the missing op/fn/hook.</t>
+          <t>op: percent_of_total (not fn: percent). op: rank. op: hook + hook: hit_rate + trailing: + value:.</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Inventing op: my_yoy. eval() in YAML. A new udfs/&lt;kpi&gt;.py. Editing core/.</t>
+          <t>fn: percent for cut share. Sorting in the host to fake rank. A window SUM for 'how often'.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>New reusable names go in capabilities/ + registries/ (How to extend sheet). Do not fake them in this KPI file.</t>
+          <t>Cut ops see the full cut. Hooks need the densified spine — declare trailing so required_span is wide enough.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="29" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Mandatory KPI keys</t>
+          <t>Map — snapshot / entity window / lookup</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>kpi_id, model, default_dimensions, ≥1 cut, ≥1 measure. time: (period) or omit entirely (snapshot). row_set span_union|anchor_only.</t>
+          <t>No period column; per-entity sequence; static code map.</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>See gold file udfs/config/kpis/sotif/3004.yaml — copy structure, not Sotif names, unless this KPI is Sotif.</t>
+          <t>Omit time:. over: on a pre-fold base (not calendar op: lag). lookup: { column, map, default }.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Missing default_dimensions. Empty measures:. cuts[].model:. parameters.selected_dimensions.</t>
+          <t>window/trend on a snapshot. Calendar op: lag for per-customer previous order. Giant CASE for a fee table.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>cuts.group_by is extras only. Header comments must name this kpi_id, not leftover 3004 text.</t>
+          <t>Snapshot leftover reporting_month skips as no_time. identity_grain required to point at a helper with no agg:.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="29" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Mandatory model keys (new extract only)</t>
+          <t>Map — cannot express</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>model_id, kind physical|sql, required_aliases, sources (physical) or sql:+output_schema (sql).</t>
+          <t>Iterative allocation, custom solver, anything with no catalog row.</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>model_id matches filename and KPI model:. SQL uses $alias_scan / $alias_path, not hardcoded URIs.</t>
+          <t>Stop. Report: cannot bind with current catalog. Name the missing op/fn/hook.</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>KPI-level sql: as the extract. A second model whose stem folds onto an existing file.</t>
+          <t>Inventing op: my_yoy. eval() in YAML. A new udfs/&lt;kpi&gt;.py. Editing core/.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Context path wins over default_paths. Prefer $alias_scan so Delta vs Parquet follows table_type.</t>
+          <t>New reusable names go in capabilities/ + registries/ (How to extend sheet). Do not fake them in this KPI file.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="29" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Completeness checklist</t>
+          <t>Mandatory KPI keys</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Emit YAML only when every box is true (same list as kpi-yaml-preparation-guide.md §0.7).</t>
+          <t>kpi_id, model, default_dimensions, ≥1 cut, ≥1 measure. time: (period) or omit entirely (snapshot). row_set span_union|anchor_only.</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Filename=kpi_id=execution.kpi_id; model matches; every host measure_key declared; every of:/expr ident exists; identifiers legal; time xor snapshot rules; no URIs; no invented names.</t>
+          <t>See gold file udfs/config/kpis/sotif/3004.yaml — copy structure, not Sotif names, unless this KPI is Sotif.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Shipping 'best effort' YAML with guessed columns. Leaving one measure_key unimplemented.</t>
+          <t>Missing default_dimensions. Empty measures:. cuts[].model:. parameters.selected_dimensions.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>If any box is false: numbered questions, no files. Closed-world names below (catalog sheets win if they disagree).</t>
+          <t>cuts.group_by is extras only. Header comments must name this kpi_id, not leftover 3004 text.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="29" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Closed-world — measure ops</t>
+          <t>Mandatory model keys (new extract only)</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>measures.op may only be one of these names (live from registries/ops.yaml).</t>
+          <t>model_id, kind physical|sql, required_aliases, sources (physical) or sql:+output_schema (sql).</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>point, window, trend, arithmetic, fn, expr, constant, dimension, predicate, hook, rank, percent_of_total, ntile, dense_rank, row_number, cumulative_share, running_total, contribution, lag, lead, index, vs_target, threshold, percent_rank, gap_to_leader, gap_to_avg, zscore, running_avg, top_n, diff, pct_change</t>
+          <t>model_id matches filename and KPI model:. SQL uses $alias_scan / $alias_path, not hardcoded URIs.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Any other op: string, including aliases you invent.</t>
+          <t>KPI-level sql: as the extract. A second model whose stem folds onto an existing file.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>See Measure ops sheet for YAML shape. Aliases listed there (if any) are the only extra spellings.</t>
+          <t>Context path wins over default_paths. Prefer $alias_scan so Delta vs Parquet follows table_type.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="29" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Closed-world — column functions</t>
+          <t>Completeness checklist</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>base_measures columns:+op: / expr call names (live from registries/functions/column.yaml).</t>
+          <t>Emit YAML only when every box is true (same list as kpi-yaml-preparation-guide.md §0.7).</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>value, abs, sum, subtract, multiply, divide, percent_of, min, max, avg, coalesce, if_null, nullif, null_if_zero, zero_if_null, is_null, is_not_null, if_else, round, floor, ceil, power, log, log10, sqrt, date_diff, date_add, epoch_day</t>
+          <t>Filename=kpi_id=execution.kpi_id; model matches; every host measure_key declared; every of:/expr ident exists; identifiers legal; time xor snapshot rules; no URIs; no invented names.</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>SQL functions that are not on this list.</t>
+          <t>Shipping 'best effort' YAML with guessed columns. Leaving one measure_key unimplemented.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>See Column functions sheet.</t>
+          <t>If any box is false: numbered questions, no files. Closed-world names below (catalog sheets win if they disagree).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="29" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Closed-world — measure functions</t>
+          <t>Closed-world — measure ops</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>op: fn / arithmetic fn: names (live from registries/functions/measure.yaml).</t>
+          <t>measures.op may only be one of these names (live from registries/ops.yaml).</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>growth_pct, divide, percent, sum, subtract, multiply, min, max, avg, abs, clamp, attainment, coalesce, if_null, nullif, null_if_zero, zero_if_null, is_null, is_not_null, if_else, sign_label, round, floor, ceil, power, log, log10, sqrt, date_diff, date_add, epoch_day</t>
+          <t>point, window, trend, arithmetic, fn, expr, constant, dimension, predicate, hook, rank, percent_of_total, ntile, dense_rank, row_number, cumulative_share, running_total, contribution, lag, lead, index, vs_target, threshold, percent_rank, gap_to_leader, gap_to_avg, zscore, running_avg, top_n, diff, pct_change</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>fn: yoy as a new name — use growth_pct (alias yoy/mom if listed on that sheet).</t>
+          <t>Any other op: string, including aliases you invent.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>See Measure functions sheet.</t>
+          <t>See Measure ops sheet for YAML shape. Aliases listed there (if any) are the only extra spellings.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="29" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Closed-world — column functions</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>base_measures columns:+op: / expr call names (live from registries/functions/column.yaml).</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>value, abs, sum, subtract, multiply, divide, percent_of, min, max, avg, coalesce, if_null, nullif, null_if_zero, zero_if_null, is_null, is_not_null, if_else, round, floor, ceil, power, log, log10, sqrt, date_diff, date_add, epoch_day</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>SQL functions that are not on this list.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>See Column functions sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="29" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Closed-world — measure functions</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>op: fn / arithmetic fn: names (live from registries/functions/measure.yaml).</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>growth_pct, divide, percent, sum, subtract, multiply, min, max, avg, abs, clamp, attainment, coalesce, if_null, nullif, null_if_zero, zero_if_null, is_null, is_not_null, if_else, sign_label, round, floor, ceil, power, log, log10, sqrt, date_diff, date_add, epoch_day</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>fn: yoy as a new name — use growth_pct (alias yoy/mom if listed on that sheet).</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>See Measure functions sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="29" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t>Closed-world — hooks</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>op: hook + hook: names (live from registries/hooks.yaml). Always declare trailing/offset so the scan is wide enough.</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>seasonal_index, ewma, period_max, period_min, period_median, period_avg, period_sum, hit_rate, streak, period_stdev, period_var, period_cv, period_range, period_count, miss_rate, miss_streak, longest_streak, cagr, slope</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>A hook name that is not listed. Using a window SUM as a substitute for hit_rate.</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>See Hooks sheet. Hooks that list requires_value need value:.</t>
         </is>
@@ -11288,7 +11371,7 @@
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Value of a base, point, or window measure at offset before the anchor.</t>
+          <t>Value of a base or shiftable measure at offset before the anchor.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -11336,7 +11419,7 @@
       <c r="D21" s="4" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Value of a base, point, or window measure at offset after the anchor.</t>
+          <t>Value of a base or shiftable measure at offset after the anchor.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -11384,7 +11467,7 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>of / lagged of × 100. 100 means unchanged vs the offset period.</t>
+          <t>of / lagged of × 100. Source is a base or shiftable measure. 100 means unchanged vs the offset period.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -11816,7 +11899,7 @@
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>of minus the same measure at offset before the anchor.</t>
+          <t>of minus the same measure at offset before the anchor. Source is a base or shiftable measure.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -11864,7 +11947,7 @@
       <c r="D32" s="5" t="inlineStr"/>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>growth_pct(of, lagged of) at offset. Same scale as fn growth_pct.</t>
+          <t>growth_pct(of, lagged of) at offset. Source is a base or shiftable measure. Same scale as fn growth_pct.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Point imports and YAML lookup at the flattened layout so Hub can set KPI_ENGINE_CONFIG_DIR and import kpi_engine.pipeline without putting the package directory on sys.path.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KPI-Engine-Capabilities.xlsx
+++ b/docs/KPI-Engine-Capabilities.xlsx
@@ -749,7 +749,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live allowlist from udfs/kpi_engine/registries/. YAML may only name what is listed here. Generated for authors, architects, and leadership.</t>
+          <t>Live allowlist from kpi_engine/registries/. YAML may only name what is listed here. Generated for authors, architects, and leadership.</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>If nothing matches: new catalog name, not core/</t>
+          <t>If nothing matches: new catalog name, not pipeline/</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Copy the pattern into config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
+          <t>Copy the pattern into kpi_config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>If no pattern fits, add a catalog name — do not edit core/</t>
+          <t>If no pattern fits, add a catalog name — do not edit pipeline/</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Host entry: udfs.kpi_engine.main   |   Routing: execution.kpi_id → config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml   |   AI brief: attach YAML preparation + catalogs + calculation intake (kpi-yaml-preparation-guide.md §0).</t>
+          <t>Host entry: kpi_engine.main   |   YAML root: KPI_ENGINE_CONFIG_DIR or sibling kpi_config/   |   Routing: execution.kpi_id → kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml   |   AI brief: attach YAML preparation + catalogs + calculation intake (kpi-yaml-preparation-guide.md §0).</t>
         </is>
       </c>
     </row>
@@ -6674,17 +6674,17 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Copy config/kpis/sotif/3004.yaml → &lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml. Fill time, dimensions, base_measures, cuts, measures. Host module_path stays udfs.kpi_engine.main.</t>
+          <t>Copy kpi_config/kpis/sotif/3004.yaml → &lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml. Fill time, dimensions, base_measures, cuts, measures. Host module_path stays kpi_engine.main.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>udfs/config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
+          <t>kpi_config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Do not add udfs/&lt;kpi&gt;.py. Do not edit core/.</t>
+          <t>Do not add a per-KPI Python module. Do not edit pipeline/.</t>
         </is>
       </c>
     </row>
@@ -6701,12 +6701,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Add config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml (kind: physical or sql). Point KPI model: at model_id. Paths stay on context.datasets.</t>
+          <t>Add kpi_config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml (kind: physical or sql). Point KPI model: at model_id. Paths stay on context.datasets.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>udfs/config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
+          <t>kpi_config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Not a core/ edit. KPI YAML uses op: &lt;new_name&gt;.</t>
+          <t>Not a pipeline/ edit. KPI YAML uses op: &lt;new_name&gt;.</t>
         </is>
       </c>
     </row>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>kpi_engine/core/ + contracts.py</t>
+          <t>kpi_engine/pipeline/ + contracts.py</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>core/filter_ops.py</t>
+          <t>pipeline/filter_ops.py</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>After any registry change, regenerate udfs/kpi_engine/registries/CAPABILITIES.md (write_generated_docs).</t>
+          <t>After any registry change, regenerate kpi_engine/registries/CAPABILITIES.md (write_generated_docs).</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>config/kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml (or flat kpis/&lt;kpi_id&gt;.yaml)</t>
+          <t>kpi_config/kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml (or flat kpis/&lt;kpi_id&gt;.yaml)</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -7038,7 +7038,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml  —  KPI model: pointer</t>
+          <t>kpi_config/models/&lt;kpi_group&gt;/&lt;id&gt;.yaml  —  KPI model: pointer</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -7422,14 +7422,14 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Extending the engine without editing core/.</t>
+          <t>Extending the engine without editing pipeline/.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>core/ (frozen pipeline)</t>
+          <t>pipeline/ (frozen pipeline)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>udfs/kpi_engine/core/</t>
+          <t>kpi_engine/pipeline/</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Path: udfs/config/kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml or flat kpis/&lt;kpi_id&gt;.yaml. Stem equals execution.kpi_id exactly (no fold). kpi_id is unique across groups.</t>
+          <t>Path: kpi_config/kpis/&lt;kpi_group&gt;/&lt;kpi_id&gt;.yaml or flat kpis/&lt;kpi_id&gt;.yaml. Stem equals execution.kpi_id exactly (no fold). kpi_id is unique across groups.</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Path: udfs/config/models/&lt;kpi_group&gt;/&lt;model_id&gt;.yaml or flat models/&lt;model_id&gt;.yaml. Prefer lowercase snake_case. Extension must be .yaml. model_id is unique across groups.</t>
+          <t>Path: kpi_config/models/&lt;kpi_group&gt;/&lt;model_id&gt;.yaml or flat models/&lt;model_id&gt;.yaml. Prefer lowercase snake_case. Extension must be .yaml. model_id is unique across groups.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -8004,17 +8004,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>One generic entry: udfs.kpi_engine.main. Routing is execution.kpi_id → config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml (or flat kpis/&lt;id&gt;.yaml). Do not add a per-KPI Python module.</t>
+          <t>One generic entry: kpi_engine.main. Routing is execution.kpi_id → kpi_config/kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml (or flat kpis/&lt;id&gt;.yaml). Do not add a per-KPI Python module.</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Host module_path: udfs.kpi_engine.main. New KPI = new YAML (+ model YAML if the extract is new).</t>
+          <t>Host module_path: kpi_engine.main. New KPI = new YAML (+ model YAML if the extract is new).</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>udfs/&lt;kpi_id&gt;/main.py. Cloning the engine per metric. A second module_path per kpi_id.</t>
+          <t>kpi_engine/&lt;kpi_id&gt;/main.py. Cloning the engine per metric. A second module_path per kpi_id.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -8063,7 +8063,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>See udfs/config/kpis/sotif/3004.yaml and udfs/config/models/sotif/sotif.yaml headers.</t>
+          <t>See kpi_config/kpis/sotif/3004.yaml and kpi_config/models/sotif/sotif.yaml headers.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -8205,7 +8205,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>See Naming conventions. .yaml only. Host module_path stays udfs.kpi_engine.main.</t>
+          <t>See Naming conventions. .yaml only. Host module_path stays kpi_engine.main.</t>
         </is>
       </c>
     </row>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Inventing op: my_yoy. eval() in YAML. A new udfs/&lt;kpi&gt;.py. Editing core/.</t>
+          <t>Inventing op: my_yoy. eval() in YAML. A per-KPI Python module. Editing pipeline/.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -8578,7 +8578,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>See gold file udfs/config/kpis/sotif/3004.yaml — copy structure, not Sotif names, unless this KPI is Sotif.</t>
+          <t>See gold file kpi_config/kpis/sotif/3004.yaml — copy structure, not Sotif names, unless this KPI is Sotif.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Editing core/ per KPI</t>
+          <t>Editing pipeline/ per KPI</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Treat time parts as independent filters so year-only and month-only requests fold a selection instead of requiring a single month.
Existing scalar filter_code KPIs keep today's numbers; output_cut on the request is now the also_emit walk root rather than a hard lock.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KPI-Engine-Capabilities.xlsx
+++ b/docs/KPI-Engine-Capabilities.xlsx
@@ -270,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="All_operations" displayName="All_operations" ref="A1:E30" headerRowCount="1">
-  <autoFilter ref="A1:E30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="All_operations" displayName="All_operations" ref="A1:E32" headerRowCount="1">
+  <autoFilter ref="A1:E32"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Operation"/>
@@ -5240,7 +5240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Bucket of the time column. Fiscal calendar only for Q/Y.</t>
+          <t>Bucket of the time column. Fiscal calendar only for Q/Y. Week is ISO-only.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -5724,20 +5724,24 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>point offset</t>
+          <t>periods year/quarter/month/week/day</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Same measure at calendar offset from anchor.</t>
+          <t>Independent predicates. Selection S = matching grain buckets; anchor = max(S). Point folds S; windows/trends from anchor.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>previous_year_value: { of: sotif_value, op: point, offset: { years: 1 } }</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr"/>
+          <t>time: { periods: { year: year, month: "current month" } }</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Cannot set with compose:. Finer than grain is a bind error.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="29" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -5747,17 +5751,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>window trailing / leading</t>
+          <t>point offset</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Inclusive trailing N (or leading) periods as one number.</t>
+          <t>Same measure over the (shifted) selection. Year-only + years:1 is the full prior year.</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>value_3m: { of: sotif_value, op: window, trailing: { months: 3 }, inclusive: true }</t>
+          <t>previous_year_value: { of: sotif_value, op: point, offset: { years: 1 } }</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
@@ -5770,22 +5774,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>window range</t>
+          <t>window trailing / leading</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>ytd, qtd, mtd, wtd, cumulative, full_month/quarter/year.</t>
+          <t>Inclusive trailing N (or leading) periods from anchor as one number.</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>value_qtd: { of: sotif_value, op: window, range: qtd }</t>
+          <t>value_3m: { of: sotif_value, op: window, trailing: { months: 3 }, inclusive: true }</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>wtd needs day grain</t>
+          <t>trailing: 3 from June is Apr-Jun</t>
         </is>
       </c>
     </row>
@@ -5797,22 +5801,22 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>trend</t>
+          <t>window range</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Fixed-length array + trend_axes / trend_labels. Cap 50,000 cells/cut.</t>
+          <t>ytd, qtd, mtd, wtd, cumulative, full_month/quarter/year. Named ranges are anchor-relative.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>trend_12m: { of: sotif_value, op: trend, trailing: { months: 12 } }</t>
+          <t>value_qtd: { of: sotif_value, op: window, range: qtd }</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Defaults to default_cut only</t>
+          <t>mtd under year=2026 is December</t>
         </is>
       </c>
     </row>
@@ -5824,49 +5828,49 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>snapshot (omit time:)</t>
+          <t>trend</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>No month filter; all matching rows. Host reporting_month skipped as no_time.</t>
+          <t>Fixed-length array + trend_axes / trend_labels. Cap 50,000 cells/cut.</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Omit the time: block; only point offset 0 (and constants).</t>
+          <t>trend_12m: { of: sotif_value, op: trend, trailing: { months: 12 } }</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>No windows/trends/nonzero offsets</t>
+          <t>Defaults to default_cut only</t>
         </is>
       </c>
     </row>
     <row r="24" ht="29" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Cuts</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>group_by / ignore_filters / also_emit</t>
+          <t>snapshot (omit time:)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Named grains. G/R are examples, not hardcoded.</t>
+          <t>No month filter; all matching rows. Host reporting_month skipped as no_time.</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>cuts: [{ name: G, group_by: [], ignore_filters: [region], also_emit: [R] }]</t>
+          <t>Omit the time: block; only point offset 0 (and constants).</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>selected_dimensions overlays request grain</t>
+          <t>No windows/trends/nonzero offsets</t>
         </is>
       </c>
     </row>
@@ -5878,22 +5882,22 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>having</t>
+          <t>group_by / ignore_filters / also_emit</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Drop groups that fail measure predicates. Optional then_group_by.</t>
+          <t>Named grains. G/R are examples, not hardcoded.</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>having: { predicates: [{ of: current_value, cmp: gt, value: 0 }] }</t>
+          <t>cuts: [{ name: G, group_by: [], ignore_filters: [region], also_emit: [R] }]</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>cmp: gt gte lt lte eq ne between</t>
+          <t>selected_dimensions overlays request grain</t>
         </is>
       </c>
     </row>
@@ -5905,124 +5909,178 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>green_when</t>
+          <t>output_cut / pack_also_emit</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Boolean green flag on survivors (above/below).</t>
+          <t>Context output_cut is the also_emit walk root. YAML default does not lock. pack_also_emit: false emits only that cut.</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>green_when: { of: current_value, above: 40 }</t>
+          <t>cuts: [{ name: G, also_emit: [R], pack_also_emit: false }]</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Does not drop rows</t>
+          <t>Declare parameters.output_cut to accept the overlay</t>
         </is>
       </c>
     </row>
     <row r="27" ht="29" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Cuts</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>apply extract / calc / result</t>
+          <t>having</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>DuckDB WHERE vs Pandas vs drop JSON rows.</t>
+          <t>Drop groups that fail measure predicates. Optional then_group_by.</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>filters: { region: { apply: extract } }</t>
+          <t>having: { predicates: [{ of: current_value, cmp: gt, value: 0 }] }</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Unmapped valued filters are FilterError</t>
+          <t>cmp: gt gte lt lte eq ne between</t>
         </is>
       </c>
     </row>
     <row r="28" ht="29" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Multi-model</t>
+          <t>Cuts</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>model_relations</t>
+          <t>green_when</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Join two extracts on declared keys.</t>
+          <t>Boolean green flag on survivors (above/below).</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>model_relations: [{ left: a, right: b, on: [event_month, region], how: left }]</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr"/>
+          <t>green_when: { of: current_value, above: 40 }</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Does not drop rows</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="29" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>identity_grain</t>
+          <t>apply extract / calc / result</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Helpers as measures.of only when every emitted cut equals this grain.</t>
+          <t>DuckDB WHERE vs Pandas vs drop JSON rows.</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>identity_grain: [carrier_id, shipment_id]</t>
+          <t>filters: { region: { apply: extract } }</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Otherwise BindError; fold with agg:</t>
+          <t>Unmapped valued filters are FilterError</t>
         </is>
       </c>
     </row>
     <row r="30" ht="29" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
+          <t>Multi-model</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>model_relations</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Join two extracts on declared keys.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>model_relations: [{ left: a, right: b, on: [event_month, region], how: left }]</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31" ht="29" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>identity_grain</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Helpers as measures.of only when every emitted cut equals this grain.</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>identity_grain: [carrier_id, shipment_id]</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Otherwise BindError; fold with agg:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="29" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t>SQL model</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>kind: sql</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Shape extract with CTEs; walked columns must be in output_schema.</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>models/&lt;id&gt;.yaml kind: sql + sql: + output_schema:</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Not KPI sql: formulas</t>
         </is>
@@ -7273,7 +7331,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>G/R are examples. group_by, ignore_filters, also_emit. Request grain overlays selected_dimensions.</t>
+          <t>G/R are examples. group_by, ignore_filters, also_emit, pack_also_emit. Request grain overlays selected_dimensions. Context output_cut is the walk root.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -7285,7 +7343,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Global avg is recomputed, never mean of regional avgs.</t>
+          <t>Global avg is recomputed, never mean of regional avgs. YAML default for output_cut does not lock.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -7955,17 +8013,17 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>filter_code: reporting_month. filter_map: { "Supplier Name": supplier_name }.</t>
+          <t>filter_code: reporting_month. periods: { year: year, month: "current month" }. filter_map: { "Supplier Name": supplier_name }.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>filter_map values with spaces or hyphens. Omitting filter_code when time: is present.</t>
+          <t>filter_map values with spaces or hyphens. Setting periods: and compose: together.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>time.filter_code is required when time: is declared. It names the context filter that carries the selected period (the anchor), not a month IN list.</t>
+          <t>time.filter_code is required unless periods: or compose: is set. A scalar filter_code on the context still wins (one period, not a month IN list). periods: parts are independent predicates.</t>
         </is>
       </c>
     </row>
@@ -8217,22 +8275,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Either time.column + grain (day|week|month|quarter|year) + filter_code, or snapshot: true (omit time:).</t>
+          <t>Either time.column + grain (day|week|month|quarter|year) plus filter_code and/or periods:, or snapshot: true (omit time:).</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>time: { column: event_month, grain: month, filter_code: reporting_month, calendar: gregorian }.</t>
+          <t>time: { column: event_month, grain: month, periods: { year: year, month: "current month" }, calendar: gregorian }.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Guessing reporting_month. execution.time_grain. Two values as a range. Defaulting to 'latest' when the filter is missing.</t>
+          <t>Guessing reporting_month. execution.time_grain. Setting periods: and compose: together. A part finer than time.grain.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>The time filter is the anchor (exactly one value), never WHERE month IN (one month). Snapshot forbids window/trend/nonzero offset.</t>
+          <t>Scalar filter_code on the context is one value and wins. periods: parts conjoin (year alone = full year). Missing parts probe history. Snapshot forbids window/trend/nonzero offset.</t>
         </is>
       </c>
     </row>
@@ -8244,7 +8302,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>dimensions (name + from physical column). default_dimensions (required, [] = worldwide). At least one cut. default_cut.</t>
+          <t>dimensions (name + from physical column). default_dimensions (required, [] = worldwide). At least one cut. default_cut. output_cut is a walk root (pack_also_emit: false locks one cut).</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -10508,7 +10566,7 @@
       <c r="D2" s="5" t="inlineStr"/>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Value at the selected period, optional calendar offset.</t>
+          <t>Value over the time selection (one bucket or many), optional calendar offset.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -11371,7 +11429,7 @@
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Value of a base or shiftable measure at offset before the anchor.</t>
+          <t>Value of a base or shiftable measure over the selection shifted by offset.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -11419,7 +11477,7 @@
       <c r="D21" s="4" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Value of a base or shiftable measure at offset after the anchor.</t>
+          <t>Value of a base or shiftable measure over the selection shifted forward by offset.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -11467,7 +11525,7 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>of / lagged of × 100. Source is a base or shiftable measure. 100 means unchanged vs the offset period.</t>
+          <t>of / lagged of × 100 over the selection vs the shifted selection. Source is a base or shiftable measure. 100 means unchanged.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -11899,7 +11957,7 @@
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>of minus the same measure at offset before the anchor. Source is a base or shiftable measure.</t>
+          <t>of minus the same measure over the selection shifted by offset. Source is a base or shiftable measure.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -11947,7 +12005,7 @@
       <c r="D32" s="5" t="inlineStr"/>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>growth_pct(of, lagged of) at offset. Source is a base or shiftable measure. Same scale as fn growth_pct.</t>
+          <t>growth_pct(of, lagged of) over the selection vs the shifted selection. Source is a base or shiftable measure. Same scale as fn growth_pct.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Close remaining calculation gaps so YAML can express stats, shiftable hooks, cut-derived math, and per-measure filters without changing existing KPIs.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KPI-Engine-Capabilities.xlsx
+++ b/docs/KPI-Engine-Capabilities.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Hooks" displayName="Hooks" ref="A1:K20" headerRowCount="1">
-  <autoFilter ref="A1:K20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Hooks" displayName="Hooks" ref="A1:K22" headerRowCount="1">
+  <autoFilter ref="A1:K22"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Role"/>
@@ -270,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="All_operations" displayName="All_operations" ref="A1:E32" headerRowCount="1">
-  <autoFilter ref="A1:E32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="All_operations" displayName="All_operations" ref="A1:E33" headerRowCount="1">
+  <autoFilter ref="A1:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Operation"/>
@@ -4197,7 +4197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4482,7 +4482,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>rolling_median</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Median of period values in the trailing window.</t>
@@ -5225,6 +5229,105 @@
       </c>
       <c r="J20" s="5" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21" ht="81" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>mad</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>addon</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Median absolute deviation of period values in the trailing window.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>robust_spread:
+  op: hook
+  hook: mad
+  of: sotif_value
+  trailing: { months: 12 }</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>measures: { op: hook, hook: &lt;name&gt;, of: &lt;base&gt;, trailing: { months: N } }. Declare trailing/offset so required_span is wide enough. Hooks that list requires_value need value:.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>kpi_engine.capabilities.hooks.impl</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>mad</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="94" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>projection</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>addon</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Linear forecast — last observed value plus slope times periods_ahead (default 1).</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>next_month:
+  op: hook
+  hook: projection
+  of: sotif_value
+  trailing: { months: 12 }
+  periods_ahead: 1</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>measures: { op: hook, hook: &lt;name&gt;, of: &lt;base&gt;, trailing: { months: N } }. Declare trailing/offset so required_span is wide enough. Hooks that list requires_value need value:.</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>kpi_engine.capabilities.hooks.impl</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>projection</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5240,7 +5343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5358,7 +5461,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="29" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Row helper</t>
@@ -5371,17 +5474,18 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Pandas row mask before fold. Numeric ops coerce the compare column. ne excludes nulls (SQL-style).</t>
+          <t>Pandas row mask before fold. Also legal on a measure whose of: is a base (clone). Numeric ops coerce the compare column. ne excludes nulls (SQL-style).</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>where: { column: mrr, op: gt, value: 0 }</t>
+          <t>where: { column: mrr, op: gt, value: 0 }
+measures.late: { of: fact, op: point, where: { column: status, op: eq, value: LATE } }</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Ops: in eq ne gt gte lt lte between. between needs values: [lo, hi]. Not like/is_null.</t>
+          <t>Ops: in eq ne gt gte lt lte between. between needs values: [lo, hi]. Not like/is_null. ignore_filters: on a measure skips context codes.</t>
         </is>
       </c>
     </row>
@@ -5470,49 +5574,49 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>first / last</t>
+          <t>stddev / variance / mode</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Identity fold after sort by time (or window). Text columns are still coerced to numeric.</t>
+          <t>Non-additive sample stdev/var (ddof=1). One row → null. mode ties → smallest.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>base_measures.bal: { sql: balance, agg: last }</t>
+          <t>base_measures.spread: { sql: amount, agg: stddev }</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Used with over: last_n</t>
+          <t>Same path as median</t>
         </is>
       </c>
     </row>
     <row r="10" ht="29" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Row helper</t>
+          <t>Aggregation</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>expr</t>
+          <t>first / last</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Named row formula on columns or earlier helpers. No DuckDB SUM().</t>
+          <t>Identity fold after sort by time (or window). Text columns are still coerced to numeric.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>gross: { expr: qty * price }</t>
+          <t>base_measures.bal: { sql: balance, agg: last }</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Add agg: to fold, or identity_grain for point of</t>
+          <t>Used with over: last_n</t>
         </is>
       </c>
     </row>
@@ -5524,20 +5628,24 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>lookup</t>
+          <t>expr</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Map a column through a dict; default or strict.</t>
+          <t>Named row formula on columns or earlier helpers. No DuckDB SUM().</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>fee: { lookup: { column: pay, map: { COD: 25 }, default: 10 } }</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
+          <t>gross: { expr: qty * price }</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Add agg: to fold, or identity_grain for point of</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="29" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -5547,17 +5655,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>sql: column</t>
+          <t>lookup</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Pass a physical column (or simple ident). Default agg is sum if omitted.</t>
+          <t>Map a column through a dict; default or strict.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>sotif_value: { sql: amount, agg: sum }</t>
+          <t>fee: { lookup: { column: pay, map: { COD: 25 }, default: 10 } }</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
@@ -5570,49 +5678,45 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>columns + op</t>
+          <t>sql: column</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Call a column function by name.</t>
+          <t>Pass a physical column (or simple ident). Default agg is sum if omitted.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>ontime_full: { columns: [ontime, fullqty], op: multiply, agg: sum }</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>See Column functions sheet</t>
-        </is>
-      </c>
+          <t>sotif_value: { sql: amount, agg: sum }</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Entity window</t>
+          <t>Row helper</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>over.lag / lead</t>
+          <t>columns + op</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Value from another row in partition, ordered by order_by. Requires of:.</t>
+          <t>Call a column function by name.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>prev: { over: { fn: lag, of: order_date, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
+          <t>ontime_full: { columns: [ontime, fullqty], op: multiply, agg: sum }</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Not calendar op: lag</t>
+          <t>See Column functions sheet</t>
         </is>
       </c>
     </row>
@@ -5624,20 +5728,24 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>over.row_number / rank / dense_rank</t>
+          <t>over.lag / lead</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Sequence in partition. of: optional.</t>
+          <t>Value from another row in partition, ordered by order_by. Requires of:.</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>seq: { over: { fn: row_number, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr"/>
+          <t>prev: { over: { fn: lag, of: order_date, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Not calendar op: lag</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="29" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -5647,17 +5755,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>over.running_sum / running_avg</t>
+          <t>over.row_number / rank / dense_rank</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Running aggregate along order_by. Requires of:.</t>
+          <t>Sequence in partition. of: optional.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>run: { over: { fn: running_sum, of: net, partition_by: [carrier_id], order_by: [start] }, agg: max }</t>
+          <t>seq: { over: { fn: row_number, partition_by: [customer_id], order_by: [order_date] }, agg: max }</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -5670,49 +5778,45 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>over.last_n</t>
+          <t>over.running_sum / running_avg</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>JSON list of last n of values. Point only; cannot feed arithmetic.</t>
+          <t>Running aggregate along order_by. Requires of:.</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>recent: { over: { fn: last_n, of: amount, n: 2, partition_by: [region], order_by: [order_id] }, agg: last }</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Dates as ISO strings</t>
-        </is>
-      </c>
+          <t>run: { over: { fn: running_sum, of: net, partition_by: [carrier_id], order_by: [start] }, agg: max }</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="29" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Entity window</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>grain day/week/month/quarter/year</t>
+          <t>over.last_n</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Bucket of the time column. Fiscal calendar only for Q/Y. Week is ISO-only.</t>
+          <t>JSON list of last n of values. Point only; cannot feed arithmetic.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>time: { column: event_month, grain: month, filter_code: reporting_month }</t>
+          <t>recent: { over: { fn: last_n, of: amount, n: 2, partition_by: [region], order_by: [order_id] }, agg: last }</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>parameters.time_grain overlay if declared</t>
+          <t>Dates as ISO strings</t>
         </is>
       </c>
     </row>
@@ -5724,22 +5828,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>periods year/quarter/month/week/day</t>
+          <t>grain day/week/month/quarter/year</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Independent predicates. Selection S = matching grain buckets; anchor = max(S). Point folds S; windows/trends from anchor.</t>
+          <t>Bucket of the time column. Fiscal calendar only for Q/Y. Week is ISO-only.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>time: { periods: { year: year, month: "current month" } }</t>
+          <t>time: { column: event_month, grain: month, filter_code: reporting_month }</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Cannot set with compose:. Finer than grain is a bind error.</t>
+          <t>parameters.time_grain overlay if declared</t>
         </is>
       </c>
     </row>
@@ -5751,20 +5855,24 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>point offset</t>
+          <t>periods year/quarter/month/week/day</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Same measure over the (shifted) selection. Year-only + years:1 is the full prior year.</t>
+          <t>Independent predicates. Selection S = matching grain buckets; anchor = max(S). Point folds S; windows/trends from anchor.</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>previous_year_value: { of: sotif_value, op: point, offset: { years: 1 } }</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
+          <t>time: { periods: { year: year, month: "current month" } }</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Cannot set with compose:. Finer than grain is a bind error.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="29" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -5774,24 +5882,20 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>window trailing / leading</t>
+          <t>point offset</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Inclusive trailing N (or leading) periods from anchor as one number.</t>
+          <t>Same measure over the (shifted) selection. Year-only + years:1 is the full prior year.</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>value_3m: { of: sotif_value, op: window, trailing: { months: 3 }, inclusive: true }</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>trailing: 3 from June is Apr-Jun</t>
-        </is>
-      </c>
+          <t>previous_year_value: { of: sotif_value, op: point, offset: { years: 1 } }</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="29" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -5801,22 +5905,22 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>window range</t>
+          <t>window trailing / leading</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>ytd, qtd, mtd, wtd, cumulative, full_month/quarter/year. Named ranges are anchor-relative.</t>
+          <t>Inclusive trailing N (or leading) periods from anchor as one number.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>value_qtd: { of: sotif_value, op: window, range: qtd }</t>
+          <t>value_3m: { of: sotif_value, op: window, trailing: { months: 3 }, inclusive: true }</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>mtd under year=2026 is December</t>
+          <t>trailing: 3 from June is Apr-Jun</t>
         </is>
       </c>
     </row>
@@ -5828,22 +5932,22 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>trend</t>
+          <t>window range</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Fixed-length array + trend_axes / trend_labels. Cap 50,000 cells/cut.</t>
+          <t>ytd, qtd, mtd, wtd, cumulative, full_month/quarter/year. Named ranges are anchor-relative.</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>trend_12m: { of: sotif_value, op: trend, trailing: { months: 12 } }</t>
+          <t>value_qtd: { of: sotif_value, op: window, range: qtd }</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Defaults to default_cut only</t>
+          <t>mtd under year=2026 is December</t>
         </is>
       </c>
     </row>
@@ -5855,49 +5959,49 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>snapshot (omit time:)</t>
+          <t>trend</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>No month filter; all matching rows. Host reporting_month skipped as no_time.</t>
+          <t>Fixed-length array + trend_axes / trend_labels. Cap 50,000 cells/cut.</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Omit the time: block; only point offset 0 (and constants).</t>
+          <t>trend_12m: { of: sotif_value, op: trend, trailing: { months: 12 } }</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>No windows/trends/nonzero offsets</t>
+          <t>Defaults to default_cut only</t>
         </is>
       </c>
     </row>
     <row r="25" ht="29" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Cuts</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>group_by / ignore_filters / also_emit</t>
+          <t>snapshot (omit time:)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Named grains. G/R are examples, not hardcoded.</t>
+          <t>No month filter; all matching rows. Host reporting_month skipped as no_time.</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>cuts: [{ name: G, group_by: [], ignore_filters: [region], also_emit: [R] }]</t>
+          <t>Omit the time: block; only point offset 0 (and constants).</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>selected_dimensions overlays request grain</t>
+          <t>No windows/trends/nonzero offsets</t>
         </is>
       </c>
     </row>
@@ -5909,22 +6013,22 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>output_cut / pack_also_emit</t>
+          <t>group_by / ignore_filters / also_emit</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Context output_cut is the also_emit walk root. YAML default does not lock. pack_also_emit: false emits only that cut.</t>
+          <t>Named grains. G/R are examples, not hardcoded.</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>cuts: [{ name: G, also_emit: [R], pack_also_emit: false }]</t>
+          <t>cuts: [{ name: G, group_by: [], ignore_filters: [region], also_emit: [R] }]</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Declare parameters.output_cut to accept the overlay</t>
+          <t>selected_dimensions overlays request grain</t>
         </is>
       </c>
     </row>
@@ -5936,22 +6040,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>having</t>
+          <t>output_cut / pack_also_emit</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Drop groups that fail measure predicates. Optional then_group_by.</t>
+          <t>Context output_cut is the also_emit walk root. YAML default does not lock. pack_also_emit: false emits only that cut.</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>having: { predicates: [{ of: current_value, cmp: gt, value: 0 }] }</t>
+          <t>cuts: [{ name: G, also_emit: [R], pack_also_emit: false }]</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>cmp: gt gte lt lte eq ne between</t>
+          <t>Declare parameters.output_cut to accept the overlay</t>
         </is>
       </c>
     </row>
@@ -5963,124 +6067,151 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>green_when</t>
+          <t>having</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Boolean green flag on survivors (above/below).</t>
+          <t>Drop groups that fail measure predicates. Optional then_group_by.</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>green_when: { of: current_value, above: 40 }</t>
+          <t>having: { predicates: [{ of: current_value, cmp: gt, value: 0 }] }</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Does not drop rows</t>
+          <t>cmp: gt gte lt lte eq ne between</t>
         </is>
       </c>
     </row>
     <row r="29" ht="29" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Cuts</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>apply extract / calc / result</t>
+          <t>green_when</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>DuckDB WHERE vs Pandas vs drop JSON rows.</t>
+          <t>Boolean green flag on survivors (above/below).</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>filters: { region: { apply: extract } }</t>
+          <t>green_when: { of: current_value, above: 40 }</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Unmapped valued filters are FilterError</t>
+          <t>Does not drop rows</t>
         </is>
       </c>
     </row>
     <row r="30" ht="29" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Multi-model</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>model_relations</t>
+          <t>apply extract / calc / result</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Join two extracts on declared keys.</t>
+          <t>DuckDB WHERE vs Pandas vs drop JSON rows.</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>model_relations: [{ left: a, right: b, on: [event_month, region], how: left }]</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr"/>
+          <t>filters: { region: { apply: extract } }</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Unmapped valued filters are FilterError</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="29" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Multi-model</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>identity_grain</t>
+          <t>model_relations</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Helpers as measures.of only when every emitted cut equals this grain.</t>
+          <t>Join two extracts on declared keys.</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>identity_grain: [carrier_id, shipment_id]</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Otherwise BindError; fold with agg:</t>
-        </is>
-      </c>
+          <t>model_relations: [{ left: a, right: b, on: [event_month, region], how: left }]</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
     </row>
     <row r="32" ht="29" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>identity_grain</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Helpers as measures.of only when every emitted cut equals this grain.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>identity_grain: [carrier_id, shipment_id]</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Otherwise BindError; fold with agg:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="29" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
           <t>SQL model</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>kind: sql</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Shape extract with CTEs; walked columns must be in output_schema.</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>models/&lt;id&gt;.yaml kind: sql + sql: + output_schema:</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>Not KPI sql: formulas</t>
         </is>
@@ -8356,7 +8487,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>SUM/COUNT/MIN/MAX of a column at the selected period.</t>
+          <t>SUM/COUNT/MIN/MAX of a column over the time selection (one bucket or many).</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -8372,7 +8503,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>agg: sum | avg | count | count_distinct | min | max | median | percentile | first | last.</t>
+          <t>agg: sum | avg | count | count_distinct | min | max | median | percentile | first | last | stddev | variance | mode.</t>
         </is>
       </c>
     </row>
@@ -8384,7 +8515,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Same metric last year/month/quarter; growth % vs that period.</t>
+          <t>Same metric last year/month/quarter over the shifted selection; growth % vs that set (year-only is year vs year).</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -8423,12 +8554,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>lag of trend/hook/rank. lag of a row helper (no agg:).</t>
+          <t>lag of trend/rank. lag of a row helper (no agg:). Rank a lagged measure instead of lagging a rank. Put offset: on the trend.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Sources: bases and shiftable measures (point, window, fn, expr, …).</t>
+          <t>Sources: bases and shiftable measures (point, window, fn, expr, hook, …).</t>
         </is>
       </c>
     </row>
@@ -8798,7 +8929,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>seasonal_index, ewma, period_max, period_min, period_median, period_avg, period_sum, hit_rate, streak, period_stdev, period_var, period_cv, period_range, period_count, miss_rate, miss_streak, longest_streak, cagr, slope</t>
+          <t>seasonal_index, ewma, period_max, period_min, period_median, period_avg, period_sum, hit_rate, streak, period_stdev, period_var, period_cv, period_range, period_count, miss_rate, miss_streak, longest_streak, cagr, slope, mad, projection</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -9146,7 +9277,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>op: percent_of_total (optional partition_by)</t>
+          <t>op: percent_of_total (optional partition_by, versus_cut)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -10242,7 +10373,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="68" customHeight="1">
+    <row r="6" ht="133" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>5. Share of worldwide (cut op)</t>
@@ -10263,7 +10394,12 @@
           <t>measures:
   group_share:
     op: percent_of_total
-    of: current_value</t>
+    of: current_value
+  vs_global:
+    op: percent_of_total
+    of: current_value
+    versus_cut: G
+    cuts: [R]</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add a compact AI YAML brief and a runtime architecture guide so authors can onboard KPIs and catalog names without loading the full prep document.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KPI-Engine-Capabilities.xlsx
+++ b/docs/KPI-Engine-Capabilities.xlsx
@@ -837,7 +837,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>kpi-yaml-preparation-guide.md §0 — do not invent ops; ask if intake is incomplete</t>
+          <t>kpi-yaml-ai-prep.md — do not invent ops; ask if intake is incomplete</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Host entry: kpi_engine.main   |   YAML root: KPI_ENGINE_CONFIG_DIR or sibling kpi_config/   |   Routing: execution.kpi_id → kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml   |   AI brief: attach YAML preparation + catalogs + calculation intake (kpi-yaml-preparation-guide.md §0).</t>
+          <t>Host entry: kpi_engine.main   |   YAML root: KPI_ENGINE_CONFIG_DIR or sibling kpi_config/   |   Routing: execution.kpi_id → kpis/&lt;kpi_group&gt;/&lt;id&gt;.yaml   |   AI brief: attach kpi-yaml-ai-prep.md + catalogs + calculation intake.</t>
         </is>
       </c>
     </row>
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Attach this workbook (Naming conventions, this sheet, Measure ops, Column/Measure functions, Hooks, YAML patterns) plus kpi-yaml-preparation-guide.md §0 plus a filled intake.</t>
+          <t>Attach this workbook (Naming conventions, this sheet, Measure ops, Column/Measure functions, Hooks, YAML patterns) plus kpi-yaml-ai-prep.md plus a filled intake.</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Emit YAML only when every box is true (same list as kpi-yaml-preparation-guide.md §0.7).</t>
+          <t>Emit YAML only when every box is true (same list as kpi-yaml-ai-prep.md §8).</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">

</xml_diff>